<commit_message>
correction des montants inversés pour le cas d acompte
</commit_message>
<xml_diff>
--- a/rapport.xlsx
+++ b/rapport.xlsx
@@ -522,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K71"/>
+  <dimension ref="A1:K94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -585,7 +585,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ANM2609BPCASDEC00014</t>
+          <t>ANM2608BPCASDEC00066</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -594,13 +594,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>-6742129.46</v>
+        <v>-65245870.54</v>
       </c>
       <c r="D2" t="b">
         <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>5448382.99</v>
+        <v>65245870.54</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
@@ -615,31 +615,31 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>5448382.99</v>
+        <v>65245870.54</v>
       </c>
       <c r="K2" t="n">
-        <v>-1293746.47</v>
+        <v>130491741.08</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ANM2608AWCASEN000067</t>
+          <t>ANM2608AWCASDEC00052</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>678249.3</v>
+        <v>-41001305.23</v>
       </c>
       <c r="D3" t="b">
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>658957.2</v>
+        <v>41001305.23</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -654,31 +654,31 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>658957.2</v>
+        <v>41001305.23</v>
       </c>
       <c r="K3" t="n">
-        <v>-19292.1</v>
+        <v>82002610.45999999</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ANM2608SGBVEN000050</t>
+          <t>ANM2608BPCASDEC00023</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>803197.02</v>
+        <v>-13746148.84</v>
       </c>
       <c r="D4" t="b">
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>793760.9399999999</v>
+        <v>13746148.84</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -693,31 +693,31 @@
         <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>793760.9399999999</v>
+        <v>13746148.84</v>
       </c>
       <c r="K4" t="n">
-        <v>-9436.08</v>
+        <v>27492297.68</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ANM2608SGOUJEN000024</t>
+          <t>ANM2608BPCASDEC00013</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>363168</v>
+        <v>-12723617.12</v>
       </c>
       <c r="D5" t="b">
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>370624</v>
+        <v>12723617.12</v>
       </c>
       <c r="F5" t="n">
         <v>0</v>
@@ -732,31 +732,31 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>370624</v>
+        <v>12723617.12</v>
       </c>
       <c r="K5" t="n">
-        <v>7456</v>
+        <v>25447234.24</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ANM2608SGTNGEN000071</t>
+          <t>ANM2608BPCASDEC00019</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>976016.8100000001</v>
+        <v>-12042309.91</v>
       </c>
       <c r="D6" t="b">
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>983242.8100000001</v>
+        <v>12042309.91</v>
       </c>
       <c r="F6" t="n">
         <v>0</v>
@@ -771,16 +771,16 @@
         <v>0</v>
       </c>
       <c r="J6" t="n">
-        <v>983242.8100000001</v>
+        <v>12042309.91</v>
       </c>
       <c r="K6" t="n">
-        <v>7226</v>
+        <v>24084619.82</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ANM2609BPCASDEC00015</t>
+          <t>ANM2608AWCASDEC00051</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -789,13 +789,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>-346461.01</v>
+        <v>-10750731.61</v>
       </c>
       <c r="D7" t="b">
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>344512.34</v>
+        <v>10750731.61</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
@@ -810,16 +810,16 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>344512.34</v>
+        <v>10750731.61</v>
       </c>
       <c r="K7" t="n">
-        <v>-1948.67</v>
+        <v>21501463.22</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ANM2608BPCASDEC00015</t>
+          <t>ANM2609BPCASDEC00014</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -828,13 +828,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>-161280</v>
+        <v>-6742129.46</v>
       </c>
       <c r="D8" t="b">
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>159876</v>
+        <v>5448382.99</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -849,16 +849,16 @@
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>159876</v>
+        <v>5448382.99</v>
       </c>
       <c r="K8" t="n">
-        <v>-1404</v>
+        <v>12190512.45</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ANM2609SGCASDEC00135</t>
+          <t>ANM2609BMCICDEC00002</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -867,13 +867,13 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>-173634.12</v>
+        <v>-5733574.23</v>
       </c>
       <c r="D9" t="b">
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>172341.31</v>
+        <v>5733574.23</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -888,16 +888,16 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>172341.31</v>
+        <v>5733574.23</v>
       </c>
       <c r="K9" t="n">
-        <v>-1292.81</v>
+        <v>11467148.46</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ANM2608BPCASDEC00065</t>
+          <t>ANM2608BPCASDEC00064</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -906,13 +906,13 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>-179267.06</v>
+        <v>-3370243.69</v>
       </c>
       <c r="D10" t="b">
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>177993.86</v>
+        <v>3370243.69</v>
       </c>
       <c r="F10" t="n">
         <v>0</v>
@@ -927,31 +927,31 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>177993.86</v>
+        <v>3370243.69</v>
       </c>
       <c r="K10" t="n">
-        <v>-1273.2</v>
+        <v>6740487.38</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ANM2608CARR2EN000180</t>
+          <t>ANM2608BPCASDEC00009</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1116.62</v>
+        <v>-2121334.19</v>
       </c>
       <c r="D11" t="b">
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>2233.24</v>
+        <v>2121334.19</v>
       </c>
       <c r="F11" t="n">
         <v>0</v>
@@ -966,31 +966,31 @@
         <v>0</v>
       </c>
       <c r="J11" t="n">
-        <v>2233.24</v>
+        <v>2121334.19</v>
       </c>
       <c r="K11" t="n">
-        <v>1116.62</v>
+        <v>4242668.38</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ANM2607SGAGEN000092</t>
+          <t>ANM2608AWCASDEC00050</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>40282.48</v>
+        <v>-1016163.35</v>
       </c>
       <c r="D12" t="b">
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>41381.88</v>
+        <v>1016163.35</v>
       </c>
       <c r="F12" t="n">
         <v>0</v>
@@ -1005,37 +1005,37 @@
         <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>41381.88</v>
+        <v>1016163.35</v>
       </c>
       <c r="K12" t="n">
-        <v>1099.4</v>
+        <v>2032326.7</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ANM2609SGFESEN000012</t>
+          <t>ANM2608BPCASDEC00052</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>297956</v>
+        <v>-868428.23</v>
       </c>
       <c r="D13" t="b">
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>296857</v>
+        <v>0</v>
       </c>
       <c r="F13" t="n">
         <v>0</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>868428.23</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -1044,31 +1044,31 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>296857</v>
+        <v>868428.23</v>
       </c>
       <c r="K13" t="n">
-        <v>-1099</v>
+        <v>1736856.46</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ANM2608SGRABEN000095</t>
+          <t>ANM2608BPCASDEC00008</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>57256.84</v>
+        <v>-636525.97</v>
       </c>
       <c r="D14" t="b">
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>59189.41</v>
+        <v>635968.0600000001</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
@@ -1080,19 +1080,19 @@
         <v>0</v>
       </c>
       <c r="I14" t="n">
-        <v>1115.95</v>
+        <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>58073.46</v>
+        <v>635968.0600000001</v>
       </c>
       <c r="K14" t="n">
-        <v>816.62</v>
+        <v>1272494.03</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ANM2608BPCASDEC00008</t>
+          <t>ANM2608BPCASDEC00060</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1101,13 +1101,13 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>-636525.97</v>
+        <v>-485172</v>
       </c>
       <c r="D15" t="b">
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>635968.0600000001</v>
+        <v>485172</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
@@ -1122,70 +1122,70 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>635968.0600000001</v>
+        <v>485172</v>
       </c>
       <c r="K15" t="n">
-        <v>-557.91</v>
+        <v>970344</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ANM2608SGTNGEN000028</t>
+          <t>ANM2608AWCASDEC00053</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>16529.06</v>
+        <v>-420846.76</v>
       </c>
       <c r="D16" t="b">
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>16367.26</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>420846.76</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
       </c>
       <c r="I16" t="n">
-        <v>338.2</v>
+        <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>16029.06</v>
+        <v>420846.76</v>
       </c>
       <c r="K16" t="n">
-        <v>-500</v>
+        <v>841693.52</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ANM2608SGAGEN000035</t>
+          <t>ANM2609BPCASDEC00015</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>22760.24</v>
+        <v>-346461.01</v>
       </c>
       <c r="D17" t="b">
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>23223.59</v>
+        <v>344512.34</v>
       </c>
       <c r="F17" t="n">
         <v>0</v>
@@ -1200,31 +1200,31 @@
         <v>0</v>
       </c>
       <c r="J17" t="n">
-        <v>23223.59</v>
+        <v>344512.34</v>
       </c>
       <c r="K17" t="n">
-        <v>463.35</v>
+        <v>690973.35</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ANM2608SGAGEN000082</t>
+          <t>ANM2608BPCASDEC00012</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>31795.58</v>
+        <v>-318600.03</v>
       </c>
       <c r="D18" t="b">
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>32255.43</v>
+        <v>318600.03</v>
       </c>
       <c r="F18" t="n">
         <v>0</v>
@@ -1239,37 +1239,37 @@
         <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>32255.43</v>
+        <v>318600.03</v>
       </c>
       <c r="K18" t="n">
-        <v>459.85</v>
+        <v>637200.0600000001</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ANM2608SGAGEN000081</t>
+          <t>ANM2608BPCASDEC00057</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>23772.23</v>
+        <v>-251625.19</v>
       </c>
       <c r="D19" t="b">
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>24231.59</v>
+        <v>0</v>
       </c>
       <c r="F19" t="n">
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>0</v>
+        <v>251625.19</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
@@ -1278,31 +1278,31 @@
         <v>0</v>
       </c>
       <c r="J19" t="n">
-        <v>24231.59</v>
+        <v>251625.19</v>
       </c>
       <c r="K19" t="n">
-        <v>459.36</v>
+        <v>503250.38</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ANM2608SGAGEN000079</t>
+          <t>ANM2608BPCASDEC00065</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>27324.59</v>
+        <v>-179267.06</v>
       </c>
       <c r="D20" t="b">
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>27779.25</v>
+        <v>177993.86</v>
       </c>
       <c r="F20" t="n">
         <v>0</v>
@@ -1317,31 +1317,31 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>27779.25</v>
+        <v>177993.86</v>
       </c>
       <c r="K20" t="n">
-        <v>454.66</v>
+        <v>357260.92</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ANM2608SGAGEN000034</t>
+          <t>ANM2609SGCASDEC00135</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>20632.11</v>
+        <v>-173634.12</v>
       </c>
       <c r="D21" t="b">
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>21075.05</v>
+        <v>172341.31</v>
       </c>
       <c r="F21" t="n">
         <v>0</v>
@@ -1356,16 +1356,16 @@
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>21075.05</v>
+        <v>172341.31</v>
       </c>
       <c r="K21" t="n">
-        <v>442.94</v>
+        <v>345975.43</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ANM2608BPCASDEC00022</t>
+          <t>ANM2608BPCASDEC00015</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1374,13 +1374,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>-48456.07</v>
+        <v>-161280</v>
       </c>
       <c r="D22" t="b">
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>48074.26</v>
+        <v>159876</v>
       </c>
       <c r="F22" t="n">
         <v>0</v>
@@ -1395,37 +1395,37 @@
         <v>0</v>
       </c>
       <c r="J22" t="n">
-        <v>48074.26</v>
+        <v>159876</v>
       </c>
       <c r="K22" t="n">
-        <v>-381.81</v>
+        <v>321156</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ANM2608SGAGEN000083</t>
+          <t>ANM2608BPCASDEC00063</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>19807.2</v>
+        <v>-112869.39</v>
       </c>
       <c r="D23" t="b">
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>20183.5</v>
+        <v>0</v>
       </c>
       <c r="F23" t="n">
         <v>0</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>112869.39</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
@@ -1434,16 +1434,16 @@
         <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>20183.5</v>
+        <v>112869.39</v>
       </c>
       <c r="K23" t="n">
-        <v>376.3</v>
+        <v>225738.78</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ANM2608BPCASDEC00014</t>
+          <t>ANM2608BPCASDEC00011</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1452,19 +1452,19 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>-76930.56</v>
+        <v>-90572.74000000001</v>
       </c>
       <c r="D24" t="b">
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>76566.37</v>
+        <v>0</v>
       </c>
       <c r="F24" t="n">
         <v>0</v>
       </c>
       <c r="G24" t="n">
-        <v>0</v>
+        <v>90572.74000000001</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
@@ -1473,31 +1473,31 @@
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>76566.37</v>
+        <v>90572.74000000001</v>
       </c>
       <c r="K24" t="n">
-        <v>-364.19</v>
+        <v>181145.48</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ANM2608SGAGEN000080</t>
+          <t>ANM2608BPCASDEC00014</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>15462.74</v>
+        <v>-76930.56</v>
       </c>
       <c r="D25" t="b">
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>15796.23</v>
+        <v>76566.37</v>
       </c>
       <c r="F25" t="n">
         <v>0</v>
@@ -1512,31 +1512,31 @@
         <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>15796.23</v>
+        <v>76566.37</v>
       </c>
       <c r="K25" t="n">
-        <v>333.49</v>
+        <v>153496.93</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ANM2608SGBVEN000036</t>
+          <t>ANM2608BPCASDEC00062</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>27277.23</v>
+        <v>-60916.36</v>
       </c>
       <c r="D26" t="b">
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>27382.71</v>
+        <v>60800.62</v>
       </c>
       <c r="F26" t="n">
         <v>0</v>
@@ -1548,34 +1548,34 @@
         <v>0</v>
       </c>
       <c r="I26" t="n">
-        <v>405.48</v>
+        <v>0</v>
       </c>
       <c r="J26" t="n">
-        <v>26977.23</v>
+        <v>60800.62</v>
       </c>
       <c r="K26" t="n">
-        <v>-300</v>
+        <v>121716.98</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ANM2608SGMKCEN000074</t>
+          <t>ANM2608BPCASDEC00056</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>132630.52</v>
+        <v>-48473.94</v>
       </c>
       <c r="D27" t="b">
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>135567.55</v>
+        <v>48473.94</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -1587,34 +1587,34 @@
         <v>0</v>
       </c>
       <c r="I27" t="n">
-        <v>3237.03</v>
+        <v>0</v>
       </c>
       <c r="J27" t="n">
-        <v>132330.52</v>
+        <v>48473.94</v>
       </c>
       <c r="K27" t="n">
-        <v>-300</v>
+        <v>96947.88</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ANM2607SGTNGEN000113</t>
+          <t>ANM2608BPCASDEC00022</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>36672.84</v>
+        <v>-48456.07</v>
       </c>
       <c r="D28" t="b">
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>37034.65</v>
+        <v>48074.26</v>
       </c>
       <c r="F28" t="n">
         <v>0</v>
@@ -1626,40 +1626,40 @@
         <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>661.8099999999999</v>
+        <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>36372.84</v>
+        <v>48074.26</v>
       </c>
       <c r="K28" t="n">
-        <v>-300</v>
+        <v>96530.33</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ANM2608SGAGEN000038</t>
+          <t>ANM2608BPCASDEC00059</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>14636.41</v>
+        <v>-47721.46</v>
       </c>
       <c r="D29" t="b">
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>14874.41</v>
+        <v>0</v>
       </c>
       <c r="F29" t="n">
         <v>0</v>
       </c>
       <c r="G29" t="n">
-        <v>0</v>
+        <v>47721.46</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
@@ -1668,31 +1668,31 @@
         <v>0</v>
       </c>
       <c r="J29" t="n">
-        <v>14874.41</v>
+        <v>47721.46</v>
       </c>
       <c r="K29" t="n">
-        <v>238</v>
+        <v>95442.92</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ANM2608SGAGEN000078</t>
+          <t>ANM2608BPCASDEC00053</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>10572.66</v>
+        <v>-29353.25</v>
       </c>
       <c r="D30" t="b">
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>10806.66</v>
+        <v>29165.74</v>
       </c>
       <c r="F30" t="n">
         <v>0</v>
@@ -1707,16 +1707,16 @@
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>10806.66</v>
+        <v>29165.74</v>
       </c>
       <c r="K30" t="n">
-        <v>234</v>
+        <v>58518.99</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ANM2608SGBVEN000041</t>
+          <t>ANM2608SGRABEN000084</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1725,13 +1725,13 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2435.42</v>
+        <v>-20000</v>
       </c>
       <c r="D31" t="b">
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>2434.31</v>
+        <v>20000</v>
       </c>
       <c r="F31" t="n">
         <v>0</v>
@@ -1740,37 +1740,37 @@
         <v>0</v>
       </c>
       <c r="H31" t="n">
-        <v>228.27</v>
+        <v>0</v>
       </c>
       <c r="I31" t="n">
-        <v>30.92</v>
+        <v>0</v>
       </c>
       <c r="J31" t="n">
-        <v>2631.66</v>
+        <v>20000</v>
       </c>
       <c r="K31" t="n">
-        <v>196.24</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ANM2608BPCASDEC00053</t>
+          <t>ANM2608AWCASEN000067</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>DECAI</t>
+          <t>ENCAI</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>-29353.25</v>
+        <v>678249.3</v>
       </c>
       <c r="D32" t="b">
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>29165.74</v>
+        <v>658957.2</v>
       </c>
       <c r="F32" t="n">
         <v>0</v>
@@ -1785,31 +1785,31 @@
         <v>0</v>
       </c>
       <c r="J32" t="n">
-        <v>29165.74</v>
+        <v>658957.2</v>
       </c>
       <c r="K32" t="n">
-        <v>-187.51</v>
+        <v>-19292.1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ANM2608SGAGEN000037</t>
+          <t>ANM2608BPCASDEC00058</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>6800.36</v>
+        <v>-8811.780000000001</v>
       </c>
       <c r="D33" t="b">
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>6987.5</v>
+        <v>8706.559999999999</v>
       </c>
       <c r="F33" t="n">
         <v>0</v>
@@ -1824,37 +1824,37 @@
         <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>6987.5</v>
+        <v>8706.559999999999</v>
       </c>
       <c r="K33" t="n">
-        <v>187.14</v>
+        <v>17518.34</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ANM2608SGAGEN000032</t>
+          <t>ANM2608BPCASDEC00021</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>10385.55</v>
+        <v>-8605.780000000001</v>
       </c>
       <c r="D34" t="b">
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>10570.71</v>
+        <v>0</v>
       </c>
       <c r="F34" t="n">
         <v>0</v>
       </c>
       <c r="G34" t="n">
-        <v>0</v>
+        <v>8605.780000000001</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
@@ -1863,37 +1863,37 @@
         <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>10570.71</v>
+        <v>8605.780000000001</v>
       </c>
       <c r="K34" t="n">
-        <v>185.16</v>
+        <v>17211.56</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ANM2607SGAGEN000091</t>
+          <t>ANM2608BPCASDEC00020</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>12007.28</v>
+        <v>-7491.29</v>
       </c>
       <c r="D35" t="b">
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>12191.46</v>
+        <v>0</v>
       </c>
       <c r="F35" t="n">
         <v>0</v>
       </c>
       <c r="G35" t="n">
-        <v>0</v>
+        <v>7491.29</v>
       </c>
       <c r="H35" t="n">
         <v>0</v>
@@ -1902,31 +1902,31 @@
         <v>0</v>
       </c>
       <c r="J35" t="n">
-        <v>12191.46</v>
+        <v>7491.29</v>
       </c>
       <c r="K35" t="n">
-        <v>184.18</v>
+        <v>14982.58</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ANM2608SGAGEN000033</t>
+          <t>ANM2609ODDI000442</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>ODDIV</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>8685.5</v>
+        <v>-7456</v>
       </c>
       <c r="D36" t="b">
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>8865.08</v>
+        <v>7456</v>
       </c>
       <c r="F36" t="n">
         <v>0</v>
@@ -1941,31 +1941,31 @@
         <v>0</v>
       </c>
       <c r="J36" t="n">
-        <v>8865.08</v>
+        <v>7456</v>
       </c>
       <c r="K36" t="n">
-        <v>179.58</v>
+        <v>14912</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ANM2607SGAGEN000090</t>
+          <t>ANM2608BPCASDEC00054</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>6851.14</v>
+        <v>-7137.98</v>
       </c>
       <c r="D37" t="b">
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>7020.6</v>
+        <v>7096.65</v>
       </c>
       <c r="F37" t="n">
         <v>0</v>
@@ -1980,31 +1980,31 @@
         <v>0</v>
       </c>
       <c r="J37" t="n">
-        <v>7020.6</v>
+        <v>7096.65</v>
       </c>
       <c r="K37" t="n">
-        <v>169.46</v>
+        <v>14234.63</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ANM2608SGAGEN000036</t>
+          <t>ANM2608BPCASDEC00016</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>11574.39</v>
+        <v>-6580.22</v>
       </c>
       <c r="D38" t="b">
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>11722.68</v>
+        <v>6553.3</v>
       </c>
       <c r="F38" t="n">
         <v>0</v>
@@ -2019,31 +2019,31 @@
         <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>11722.68</v>
+        <v>6553.3</v>
       </c>
       <c r="K38" t="n">
-        <v>148.29</v>
+        <v>13133.52</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ANM2608BPCASDEC00062</t>
+          <t>ANM2608SGBVEN000050</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>DECAI</t>
+          <t>ENCAI</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>-60916.36</v>
+        <v>803197.02</v>
       </c>
       <c r="D39" t="b">
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>60800.62</v>
+        <v>793760.9399999999</v>
       </c>
       <c r="F39" t="n">
         <v>0</v>
@@ -2058,31 +2058,31 @@
         <v>0</v>
       </c>
       <c r="J39" t="n">
-        <v>60800.62</v>
+        <v>793760.9399999999</v>
       </c>
       <c r="K39" t="n">
-        <v>-115.74</v>
+        <v>-9436.08</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ANM2608BPCASDEC00058</t>
+          <t>ANM2608SGOUJEN000024</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>DECAI</t>
+          <t>ENCAI</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>-8811.780000000001</v>
+        <v>363168</v>
       </c>
       <c r="D40" t="b">
         <v>1</v>
       </c>
       <c r="E40" t="n">
-        <v>8706.559999999999</v>
+        <v>370624</v>
       </c>
       <c r="F40" t="n">
         <v>0</v>
@@ -2097,16 +2097,16 @@
         <v>0</v>
       </c>
       <c r="J40" t="n">
-        <v>8706.559999999999</v>
+        <v>370624</v>
       </c>
       <c r="K40" t="n">
-        <v>-105.22</v>
+        <v>7456</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ANM2608SGBVEN000022</t>
+          <t>ANM2608SGTNGEN000071</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2115,13 +2115,13 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>7170.38</v>
+        <v>976016.8100000001</v>
       </c>
       <c r="D41" t="b">
         <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>7069.58</v>
+        <v>983242.8100000001</v>
       </c>
       <c r="F41" t="n">
         <v>0</v>
@@ -2136,31 +2136,31 @@
         <v>0</v>
       </c>
       <c r="J41" t="n">
-        <v>7069.58</v>
+        <v>983242.8100000001</v>
       </c>
       <c r="K41" t="n">
-        <v>-100.8</v>
+        <v>7226</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ANM2608SGAGEN000077</t>
+          <t>ANM2608BPCASDEC00055</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ENCAI</t>
+          <t>DECAI</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>4254.82</v>
+        <v>-3228.36</v>
       </c>
       <c r="D42" t="b">
         <v>1</v>
       </c>
       <c r="E42" t="n">
-        <v>4339.34</v>
+        <v>3217.98</v>
       </c>
       <c r="F42" t="n">
         <v>0</v>
@@ -2175,16 +2175,16 @@
         <v>0</v>
       </c>
       <c r="J42" t="n">
-        <v>4339.34</v>
+        <v>3217.98</v>
       </c>
       <c r="K42" t="n">
-        <v>84.52</v>
+        <v>6446.34</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ANM2608BPCASEN000088</t>
+          <t>ANM2608CARR2EN000180</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2193,13 +2193,13 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>299.99</v>
+        <v>1116.62</v>
       </c>
       <c r="D43" t="b">
         <v>1</v>
       </c>
       <c r="E43" t="n">
-        <v>229.99</v>
+        <v>2233.24</v>
       </c>
       <c r="F43" t="n">
         <v>0</v>
@@ -2214,31 +2214,31 @@
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>229.99</v>
+        <v>2233.24</v>
       </c>
       <c r="K43" t="n">
-        <v>-70</v>
+        <v>1116.62</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ANM2608BPCASDEC00054</t>
+          <t>ANM2607SGAGEN000092</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>DECAI</t>
+          <t>ENCAI</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>-7137.98</v>
+        <v>40282.48</v>
       </c>
       <c r="D44" t="b">
         <v>1</v>
       </c>
       <c r="E44" t="n">
-        <v>7096.65</v>
+        <v>41381.88</v>
       </c>
       <c r="F44" t="n">
         <v>0</v>
@@ -2253,16 +2253,16 @@
         <v>0</v>
       </c>
       <c r="J44" t="n">
-        <v>7096.65</v>
+        <v>41381.88</v>
       </c>
       <c r="K44" t="n">
-        <v>-41.33</v>
+        <v>1099.4</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ANM2608SGCASEN000111</t>
+          <t>ANM2609SGFESEN000012</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2271,16 +2271,16 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1977524.27</v>
+        <v>297956</v>
       </c>
       <c r="D45" t="b">
         <v>1</v>
       </c>
       <c r="E45" t="n">
-        <v>1384873.47</v>
+        <v>296857</v>
       </c>
       <c r="F45" t="n">
-        <v>592618.2</v>
+        <v>0</v>
       </c>
       <c r="G45" t="n">
         <v>0</v>
@@ -2292,31 +2292,31 @@
         <v>0</v>
       </c>
       <c r="J45" t="n">
-        <v>1977491.67</v>
+        <v>296857</v>
       </c>
       <c r="K45" t="n">
-        <v>-32.6</v>
+        <v>-1099</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ANM2608BPCASDEC00016</t>
+          <t>ANM2608SGRABEN000095</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>DECAI</t>
+          <t>ENCAI</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>-6580.22</v>
+        <v>57256.84</v>
       </c>
       <c r="D46" t="b">
         <v>1</v>
       </c>
       <c r="E46" t="n">
-        <v>6553.3</v>
+        <v>59189.41</v>
       </c>
       <c r="F46" t="n">
         <v>0</v>
@@ -2328,19 +2328,19 @@
         <v>0</v>
       </c>
       <c r="I46" t="n">
-        <v>0</v>
+        <v>1115.95</v>
       </c>
       <c r="J46" t="n">
-        <v>6553.3</v>
+        <v>58073.46</v>
       </c>
       <c r="K46" t="n">
-        <v>-26.92</v>
+        <v>816.62</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ANM2608SGFESEN000003</t>
+          <t>ANM2608SGTNGEN000028</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2349,13 +2349,13 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>364357</v>
+        <v>16529.06</v>
       </c>
       <c r="D47" t="b">
         <v>1</v>
       </c>
       <c r="E47" t="n">
-        <v>364333.74</v>
+        <v>16367.26</v>
       </c>
       <c r="F47" t="n">
         <v>0</v>
@@ -2367,34 +2367,34 @@
         <v>0</v>
       </c>
       <c r="I47" t="n">
-        <v>0</v>
+        <v>338.2</v>
       </c>
       <c r="J47" t="n">
-        <v>364333.74</v>
+        <v>16029.06</v>
       </c>
       <c r="K47" t="n">
-        <v>-23.26</v>
+        <v>-500</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ANM2608BPCASDEC00055</t>
+          <t>ANM2608SGAGEN000035</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>DECAI</t>
+          <t>ENCAI</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>-3228.36</v>
+        <v>22760.24</v>
       </c>
       <c r="D48" t="b">
         <v>1</v>
       </c>
       <c r="E48" t="n">
-        <v>3217.98</v>
+        <v>23223.59</v>
       </c>
       <c r="F48" t="n">
         <v>0</v>
@@ -2409,16 +2409,16 @@
         <v>0</v>
       </c>
       <c r="J48" t="n">
-        <v>3217.98</v>
+        <v>23223.59</v>
       </c>
       <c r="K48" t="n">
-        <v>-10.38</v>
+        <v>463.35</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ANM2608AWCASEN000050</t>
+          <t>ANM2608SGAGEN000082</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2427,13 +2427,13 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>560400</v>
+        <v>31795.58</v>
       </c>
       <c r="D49" t="b">
         <v>1</v>
       </c>
       <c r="E49" t="n">
-        <v>560405.92</v>
+        <v>32255.43</v>
       </c>
       <c r="F49" t="n">
         <v>0</v>
@@ -2448,16 +2448,16 @@
         <v>0</v>
       </c>
       <c r="J49" t="n">
-        <v>560405.92</v>
+        <v>32255.43</v>
       </c>
       <c r="K49" t="n">
-        <v>5.92</v>
+        <v>459.85</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ANM2608SGRABEN000110</t>
+          <t>ANM2608SGAGEN000081</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2466,13 +2466,13 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1301434.95</v>
+        <v>23772.23</v>
       </c>
       <c r="D50" t="b">
         <v>1</v>
       </c>
       <c r="E50" t="n">
-        <v>1301436.21</v>
+        <v>24231.59</v>
       </c>
       <c r="F50" t="n">
         <v>0</v>
@@ -2487,16 +2487,16 @@
         <v>0</v>
       </c>
       <c r="J50" t="n">
-        <v>1301436.21</v>
+        <v>24231.59</v>
       </c>
       <c r="K50" t="n">
-        <v>1.26</v>
+        <v>459.36</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ANM2608SGRABEN000028</t>
+          <t>ANM2608SGAGEN000079</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2505,13 +2505,13 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>69673.2</v>
+        <v>27324.59</v>
       </c>
       <c r="D51" t="b">
         <v>1</v>
       </c>
       <c r="E51" t="n">
-        <v>69674.45</v>
+        <v>27779.25</v>
       </c>
       <c r="F51" t="n">
         <v>0</v>
@@ -2526,16 +2526,16 @@
         <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>69674.45</v>
+        <v>27779.25</v>
       </c>
       <c r="K51" t="n">
-        <v>1.25</v>
+        <v>454.66</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ANM2608SGRABEN000027</t>
+          <t>ANM2608SGAGEN000034</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2544,13 +2544,13 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>571557.99</v>
+        <v>20632.11</v>
       </c>
       <c r="D52" t="b">
         <v>1</v>
       </c>
       <c r="E52" t="n">
-        <v>571559.1899999999</v>
+        <v>21075.05</v>
       </c>
       <c r="F52" t="n">
         <v>0</v>
@@ -2565,16 +2565,16 @@
         <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>571559.1899999999</v>
+        <v>21075.05</v>
       </c>
       <c r="K52" t="n">
-        <v>1.2</v>
+        <v>442.94</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ANM2608SGOUJEN000057</t>
+          <t>ANM2608SGAGEN000083</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2583,13 +2583,13 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>688728.45</v>
+        <v>19807.2</v>
       </c>
       <c r="D53" t="b">
         <v>1</v>
       </c>
       <c r="E53" t="n">
-        <v>688729.45</v>
+        <v>20183.5</v>
       </c>
       <c r="F53" t="n">
         <v>0</v>
@@ -2604,16 +2604,16 @@
         <v>0</v>
       </c>
       <c r="J53" t="n">
-        <v>688729.45</v>
+        <v>20183.5</v>
       </c>
       <c r="K53" t="n">
-        <v>1</v>
+        <v>376.3</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ANM2608BPCASEN000100</t>
+          <t>ANM2608SGAGEN000080</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2622,13 +2622,13 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>7225</v>
+        <v>15462.74</v>
       </c>
       <c r="D54" t="b">
         <v>1</v>
       </c>
       <c r="E54" t="n">
-        <v>7226</v>
+        <v>15796.23</v>
       </c>
       <c r="F54" t="n">
         <v>0</v>
@@ -2643,16 +2643,16 @@
         <v>0</v>
       </c>
       <c r="J54" t="n">
-        <v>7226</v>
+        <v>15796.23</v>
       </c>
       <c r="K54" t="n">
-        <v>1</v>
+        <v>333.49</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ANM2608BPCASEN000096</t>
+          <t>ANM2608SGBVEN000036</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2661,13 +2661,13 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>76900</v>
+        <v>27277.23</v>
       </c>
       <c r="D55" t="b">
         <v>1</v>
       </c>
       <c r="E55" t="n">
-        <v>76901</v>
+        <v>27382.71</v>
       </c>
       <c r="F55" t="n">
         <v>0</v>
@@ -2679,19 +2679,19 @@
         <v>0</v>
       </c>
       <c r="I55" t="n">
-        <v>0</v>
+        <v>405.48</v>
       </c>
       <c r="J55" t="n">
-        <v>76901</v>
+        <v>26977.23</v>
       </c>
       <c r="K55" t="n">
-        <v>1</v>
+        <v>-300</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ANM2608SGRABEN000099</t>
+          <t>ANM2607SGTNGEN000113</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2700,13 +2700,13 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>3073.39</v>
+        <v>36672.84</v>
       </c>
       <c r="D56" t="b">
         <v>1</v>
       </c>
       <c r="E56" t="n">
-        <v>3074.39</v>
+        <v>37034.65</v>
       </c>
       <c r="F56" t="n">
         <v>0</v>
@@ -2718,19 +2718,19 @@
         <v>0</v>
       </c>
       <c r="I56" t="n">
-        <v>0</v>
+        <v>661.8099999999999</v>
       </c>
       <c r="J56" t="n">
-        <v>3074.39</v>
+        <v>36372.84</v>
       </c>
       <c r="K56" t="n">
-        <v>1</v>
+        <v>-300</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ANM2608SGOUJEN000030</t>
+          <t>ANM2608SGMKCEN000074</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2739,13 +2739,13 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>161397</v>
+        <v>132630.52</v>
       </c>
       <c r="D57" t="b">
         <v>1</v>
       </c>
       <c r="E57" t="n">
-        <v>161398</v>
+        <v>135567.55</v>
       </c>
       <c r="F57" t="n">
         <v>0</v>
@@ -2757,19 +2757,19 @@
         <v>0</v>
       </c>
       <c r="I57" t="n">
-        <v>0</v>
+        <v>3237.03</v>
       </c>
       <c r="J57" t="n">
-        <v>161398</v>
+        <v>132330.52</v>
       </c>
       <c r="K57" t="n">
-        <v>1</v>
+        <v>-300</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ANM2608SGRABEN000053</t>
+          <t>ANM2608SGAGEN000038</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2778,19 +2778,19 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>38396.69</v>
+        <v>14636.41</v>
       </c>
       <c r="D58" t="b">
         <v>1</v>
       </c>
       <c r="E58" t="n">
-        <v>24900.63</v>
+        <v>14874.41</v>
       </c>
       <c r="F58" t="n">
         <v>0</v>
       </c>
       <c r="G58" t="n">
-        <v>13497</v>
+        <v>0</v>
       </c>
       <c r="H58" t="n">
         <v>0</v>
@@ -2799,16 +2799,16 @@
         <v>0</v>
       </c>
       <c r="J58" t="n">
-        <v>38397.63</v>
+        <v>14874.41</v>
       </c>
       <c r="K58" t="n">
-        <v>0.9399999999999999</v>
+        <v>238</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>ANM2608SGCASEN000100</t>
+          <t>ANM2608SGAGEN000078</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2817,13 +2817,13 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>778780.1</v>
+        <v>10572.66</v>
       </c>
       <c r="D59" t="b">
         <v>1</v>
       </c>
       <c r="E59" t="n">
-        <v>778780.8100000001</v>
+        <v>10806.66</v>
       </c>
       <c r="F59" t="n">
         <v>0</v>
@@ -2838,16 +2838,16 @@
         <v>0</v>
       </c>
       <c r="J59" t="n">
-        <v>778780.8100000001</v>
+        <v>10806.66</v>
       </c>
       <c r="K59" t="n">
-        <v>0.71</v>
+        <v>234</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ANM2608AWCASEN000010</t>
+          <t>ANM2608SGBVEN000041</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2856,13 +2856,13 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>481808</v>
+        <v>2435.42</v>
       </c>
       <c r="D60" t="b">
         <v>1</v>
       </c>
       <c r="E60" t="n">
-        <v>481808.62</v>
+        <v>2434.31</v>
       </c>
       <c r="F60" t="n">
         <v>0</v>
@@ -2871,22 +2871,22 @@
         <v>0</v>
       </c>
       <c r="H60" t="n">
-        <v>0</v>
+        <v>228.27</v>
       </c>
       <c r="I60" t="n">
-        <v>0</v>
+        <v>30.92</v>
       </c>
       <c r="J60" t="n">
-        <v>481808.62</v>
+        <v>2631.66</v>
       </c>
       <c r="K60" t="n">
-        <v>0.62</v>
+        <v>196.24</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ANM2608SGBVEN000056</t>
+          <t>ANM2608SGAGEN000037</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2895,13 +2895,13 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1357209.94</v>
+        <v>6800.36</v>
       </c>
       <c r="D61" t="b">
         <v>1</v>
       </c>
       <c r="E61" t="n">
-        <v>1357210.56</v>
+        <v>6987.5</v>
       </c>
       <c r="F61" t="n">
         <v>0</v>
@@ -2916,16 +2916,16 @@
         <v>0</v>
       </c>
       <c r="J61" t="n">
-        <v>1357210.56</v>
+        <v>6987.5</v>
       </c>
       <c r="K61" t="n">
-        <v>0.62</v>
+        <v>187.14</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ANM2608CAROUEN000115</t>
+          <t>ANM2608SGAGEN000032</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2934,13 +2934,13 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>9648</v>
+        <v>10385.55</v>
       </c>
       <c r="D62" t="b">
         <v>1</v>
       </c>
       <c r="E62" t="n">
-        <v>9648.41</v>
+        <v>10570.71</v>
       </c>
       <c r="F62" t="n">
         <v>0</v>
@@ -2955,16 +2955,16 @@
         <v>0</v>
       </c>
       <c r="J62" t="n">
-        <v>9648.41</v>
+        <v>10570.71</v>
       </c>
       <c r="K62" t="n">
-        <v>0.41</v>
+        <v>185.16</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ANM2608SGCASEN000239</t>
+          <t>ANM2607SGAGEN000091</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2973,13 +2973,13 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1647.83</v>
+        <v>12007.28</v>
       </c>
       <c r="D63" t="b">
         <v>1</v>
       </c>
       <c r="E63" t="n">
-        <v>1648.17</v>
+        <v>12191.46</v>
       </c>
       <c r="F63" t="n">
         <v>0</v>
@@ -2994,16 +2994,16 @@
         <v>0</v>
       </c>
       <c r="J63" t="n">
-        <v>1648.17</v>
+        <v>12191.46</v>
       </c>
       <c r="K63" t="n">
-        <v>0.34</v>
+        <v>184.18</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ANM2608SGMKCEN000016</t>
+          <t>ANM2608SGAGEN000033</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3012,13 +3012,13 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>75635.78</v>
+        <v>8685.5</v>
       </c>
       <c r="D64" t="b">
         <v>1</v>
       </c>
       <c r="E64" t="n">
-        <v>77106.7</v>
+        <v>8865.08</v>
       </c>
       <c r="F64" t="n">
         <v>0</v>
@@ -3030,19 +3030,19 @@
         <v>0</v>
       </c>
       <c r="I64" t="n">
-        <v>1470.59</v>
+        <v>0</v>
       </c>
       <c r="J64" t="n">
-        <v>75636.11</v>
+        <v>8865.08</v>
       </c>
       <c r="K64" t="n">
-        <v>0.33</v>
+        <v>179.58</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ANM2608SGRBYEN000020</t>
+          <t>ANM2607SGAGEN000090</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3051,13 +3051,13 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>7219.61</v>
+        <v>6851.14</v>
       </c>
       <c r="D65" t="b">
         <v>1</v>
       </c>
       <c r="E65" t="n">
-        <v>7311.61</v>
+        <v>7020.6</v>
       </c>
       <c r="F65" t="n">
         <v>0</v>
@@ -3069,19 +3069,19 @@
         <v>0</v>
       </c>
       <c r="I65" t="n">
-        <v>91.7</v>
+        <v>0</v>
       </c>
       <c r="J65" t="n">
-        <v>7219.91</v>
+        <v>7020.6</v>
       </c>
       <c r="K65" t="n">
-        <v>0.3</v>
+        <v>169.46</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ANM2608SGOUJEN000033</t>
+          <t>ANM2608SGAGEN000036</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -3090,13 +3090,13 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>973994.78</v>
+        <v>11574.39</v>
       </c>
       <c r="D66" t="b">
         <v>1</v>
       </c>
       <c r="E66" t="n">
-        <v>973994.98</v>
+        <v>11722.68</v>
       </c>
       <c r="F66" t="n">
         <v>0</v>
@@ -3111,16 +3111,16 @@
         <v>0</v>
       </c>
       <c r="J66" t="n">
-        <v>973994.98</v>
+        <v>11722.68</v>
       </c>
       <c r="K66" t="n">
-        <v>0.2</v>
+        <v>148.29</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ANM2608CARTGEN000068</t>
+          <t>ANM2608SGBVEN000022</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3129,13 +3129,13 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>8613</v>
+        <v>7170.38</v>
       </c>
       <c r="D67" t="b">
         <v>1</v>
       </c>
       <c r="E67" t="n">
-        <v>8613.15</v>
+        <v>7069.58</v>
       </c>
       <c r="F67" t="n">
         <v>0</v>
@@ -3150,16 +3150,16 @@
         <v>0</v>
       </c>
       <c r="J67" t="n">
-        <v>8613.15</v>
+        <v>7069.58</v>
       </c>
       <c r="K67" t="n">
-        <v>0.15</v>
+        <v>-100.8</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ANM2608AWCASEN000096</t>
+          <t>ANM2608SGAGEN000077</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3168,13 +3168,13 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>623516</v>
+        <v>4254.82</v>
       </c>
       <c r="D68" t="b">
         <v>1</v>
       </c>
       <c r="E68" t="n">
-        <v>623516.1</v>
+        <v>4339.34</v>
       </c>
       <c r="F68" t="n">
         <v>0</v>
@@ -3189,16 +3189,16 @@
         <v>0</v>
       </c>
       <c r="J68" t="n">
-        <v>623516.1</v>
+        <v>4339.34</v>
       </c>
       <c r="K68" t="n">
-        <v>0.1</v>
+        <v>84.52</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ANM2608CARR2EN000114</t>
+          <t>ANM2608BPCASEN000088</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3207,13 +3207,13 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>404.21</v>
+        <v>299.99</v>
       </c>
       <c r="D69" t="b">
         <v>1</v>
       </c>
       <c r="E69" t="n">
-        <v>404.28</v>
+        <v>229.99</v>
       </c>
       <c r="F69" t="n">
         <v>0</v>
@@ -3228,16 +3228,16 @@
         <v>0</v>
       </c>
       <c r="J69" t="n">
-        <v>404.28</v>
+        <v>229.99</v>
       </c>
       <c r="K69" t="n">
-        <v>0.07000000000000001</v>
+        <v>-70</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ANM2608SGBVEN000039</t>
+          <t>ANM2608SGCASEN000111</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3246,16 +3246,16 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>19350.79</v>
+        <v>1977524.27</v>
       </c>
       <c r="D70" t="b">
         <v>1</v>
       </c>
       <c r="E70" t="n">
-        <v>19596.57</v>
+        <v>1384873.47</v>
       </c>
       <c r="F70" t="n">
-        <v>0</v>
+        <v>592618.2</v>
       </c>
       <c r="G70" t="n">
         <v>0</v>
@@ -3264,51 +3264,948 @@
         <v>0</v>
       </c>
       <c r="I70" t="n">
-        <v>245.74</v>
+        <v>0</v>
       </c>
       <c r="J70" t="n">
-        <v>19350.83</v>
+        <v>1977491.67</v>
       </c>
       <c r="K70" t="n">
-        <v>0.04</v>
+        <v>-32.6</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
+          <t>ANM2608SGFESEN000003</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>364357</v>
+      </c>
+      <c r="D71" t="b">
+        <v>1</v>
+      </c>
+      <c r="E71" t="n">
+        <v>364333.74</v>
+      </c>
+      <c r="F71" t="n">
+        <v>0</v>
+      </c>
+      <c r="G71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" t="n">
+        <v>0</v>
+      </c>
+      <c r="I71" t="n">
+        <v>0</v>
+      </c>
+      <c r="J71" t="n">
+        <v>364333.74</v>
+      </c>
+      <c r="K71" t="n">
+        <v>-23.26</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>ANM2608AWCASEN000050</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>560400</v>
+      </c>
+      <c r="D72" t="b">
+        <v>1</v>
+      </c>
+      <c r="E72" t="n">
+        <v>560405.92</v>
+      </c>
+      <c r="F72" t="n">
+        <v>0</v>
+      </c>
+      <c r="G72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" t="n">
+        <v>0</v>
+      </c>
+      <c r="I72" t="n">
+        <v>0</v>
+      </c>
+      <c r="J72" t="n">
+        <v>560405.92</v>
+      </c>
+      <c r="K72" t="n">
+        <v>5.92</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>ANM2608SGRABEN000110</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>1301434.95</v>
+      </c>
+      <c r="D73" t="b">
+        <v>1</v>
+      </c>
+      <c r="E73" t="n">
+        <v>1301436.21</v>
+      </c>
+      <c r="F73" t="n">
+        <v>0</v>
+      </c>
+      <c r="G73" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" t="n">
+        <v>0</v>
+      </c>
+      <c r="I73" t="n">
+        <v>0</v>
+      </c>
+      <c r="J73" t="n">
+        <v>1301436.21</v>
+      </c>
+      <c r="K73" t="n">
+        <v>1.26</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>ANM2608SGRABEN000028</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>69673.2</v>
+      </c>
+      <c r="D74" t="b">
+        <v>1</v>
+      </c>
+      <c r="E74" t="n">
+        <v>69674.45</v>
+      </c>
+      <c r="F74" t="n">
+        <v>0</v>
+      </c>
+      <c r="G74" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" t="n">
+        <v>0</v>
+      </c>
+      <c r="I74" t="n">
+        <v>0</v>
+      </c>
+      <c r="J74" t="n">
+        <v>69674.45</v>
+      </c>
+      <c r="K74" t="n">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>ANM2608SGRABEN000027</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>571557.99</v>
+      </c>
+      <c r="D75" t="b">
+        <v>1</v>
+      </c>
+      <c r="E75" t="n">
+        <v>571559.1899999999</v>
+      </c>
+      <c r="F75" t="n">
+        <v>0</v>
+      </c>
+      <c r="G75" t="n">
+        <v>0</v>
+      </c>
+      <c r="H75" t="n">
+        <v>0</v>
+      </c>
+      <c r="I75" t="n">
+        <v>0</v>
+      </c>
+      <c r="J75" t="n">
+        <v>571559.1899999999</v>
+      </c>
+      <c r="K75" t="n">
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>ANM2608SGOUJEN000057</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>688728.45</v>
+      </c>
+      <c r="D76" t="b">
+        <v>1</v>
+      </c>
+      <c r="E76" t="n">
+        <v>688729.45</v>
+      </c>
+      <c r="F76" t="n">
+        <v>0</v>
+      </c>
+      <c r="G76" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" t="n">
+        <v>0</v>
+      </c>
+      <c r="I76" t="n">
+        <v>0</v>
+      </c>
+      <c r="J76" t="n">
+        <v>688729.45</v>
+      </c>
+      <c r="K76" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>ANM2608SGRABEN000099</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>3073.39</v>
+      </c>
+      <c r="D77" t="b">
+        <v>1</v>
+      </c>
+      <c r="E77" t="n">
+        <v>3074.39</v>
+      </c>
+      <c r="F77" t="n">
+        <v>0</v>
+      </c>
+      <c r="G77" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" t="n">
+        <v>0</v>
+      </c>
+      <c r="I77" t="n">
+        <v>0</v>
+      </c>
+      <c r="J77" t="n">
+        <v>3074.39</v>
+      </c>
+      <c r="K77" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>ANM2608BPCASEN000096</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>76900</v>
+      </c>
+      <c r="D78" t="b">
+        <v>1</v>
+      </c>
+      <c r="E78" t="n">
+        <v>76901</v>
+      </c>
+      <c r="F78" t="n">
+        <v>0</v>
+      </c>
+      <c r="G78" t="n">
+        <v>0</v>
+      </c>
+      <c r="H78" t="n">
+        <v>0</v>
+      </c>
+      <c r="I78" t="n">
+        <v>0</v>
+      </c>
+      <c r="J78" t="n">
+        <v>76901</v>
+      </c>
+      <c r="K78" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>ANM2608SGOUJEN000030</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>161397</v>
+      </c>
+      <c r="D79" t="b">
+        <v>1</v>
+      </c>
+      <c r="E79" t="n">
+        <v>161398</v>
+      </c>
+      <c r="F79" t="n">
+        <v>0</v>
+      </c>
+      <c r="G79" t="n">
+        <v>0</v>
+      </c>
+      <c r="H79" t="n">
+        <v>0</v>
+      </c>
+      <c r="I79" t="n">
+        <v>0</v>
+      </c>
+      <c r="J79" t="n">
+        <v>161398</v>
+      </c>
+      <c r="K79" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>ANM2608BPCASEN000100</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>7225</v>
+      </c>
+      <c r="D80" t="b">
+        <v>1</v>
+      </c>
+      <c r="E80" t="n">
+        <v>7226</v>
+      </c>
+      <c r="F80" t="n">
+        <v>0</v>
+      </c>
+      <c r="G80" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" t="n">
+        <v>0</v>
+      </c>
+      <c r="I80" t="n">
+        <v>0</v>
+      </c>
+      <c r="J80" t="n">
+        <v>7226</v>
+      </c>
+      <c r="K80" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>ANM2608SGRABEN000053</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>38396.69</v>
+      </c>
+      <c r="D81" t="b">
+        <v>1</v>
+      </c>
+      <c r="E81" t="n">
+        <v>24900.63</v>
+      </c>
+      <c r="F81" t="n">
+        <v>0</v>
+      </c>
+      <c r="G81" t="n">
+        <v>13497</v>
+      </c>
+      <c r="H81" t="n">
+        <v>0</v>
+      </c>
+      <c r="I81" t="n">
+        <v>0</v>
+      </c>
+      <c r="J81" t="n">
+        <v>38397.63</v>
+      </c>
+      <c r="K81" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>ANM2608SGCASEN000100</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>778780.1</v>
+      </c>
+      <c r="D82" t="b">
+        <v>1</v>
+      </c>
+      <c r="E82" t="n">
+        <v>778780.8100000001</v>
+      </c>
+      <c r="F82" t="n">
+        <v>0</v>
+      </c>
+      <c r="G82" t="n">
+        <v>0</v>
+      </c>
+      <c r="H82" t="n">
+        <v>0</v>
+      </c>
+      <c r="I82" t="n">
+        <v>0</v>
+      </c>
+      <c r="J82" t="n">
+        <v>778780.8100000001</v>
+      </c>
+      <c r="K82" t="n">
+        <v>0.71</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>ANM2608SGBVEN000056</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>1357209.94</v>
+      </c>
+      <c r="D83" t="b">
+        <v>1</v>
+      </c>
+      <c r="E83" t="n">
+        <v>1357210.56</v>
+      </c>
+      <c r="F83" t="n">
+        <v>0</v>
+      </c>
+      <c r="G83" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" t="n">
+        <v>0</v>
+      </c>
+      <c r="I83" t="n">
+        <v>0</v>
+      </c>
+      <c r="J83" t="n">
+        <v>1357210.56</v>
+      </c>
+      <c r="K83" t="n">
+        <v>0.62</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>ANM2608AWCASEN000010</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>481808</v>
+      </c>
+      <c r="D84" t="b">
+        <v>1</v>
+      </c>
+      <c r="E84" t="n">
+        <v>481808.62</v>
+      </c>
+      <c r="F84" t="n">
+        <v>0</v>
+      </c>
+      <c r="G84" t="n">
+        <v>0</v>
+      </c>
+      <c r="H84" t="n">
+        <v>0</v>
+      </c>
+      <c r="I84" t="n">
+        <v>0</v>
+      </c>
+      <c r="J84" t="n">
+        <v>481808.62</v>
+      </c>
+      <c r="K84" t="n">
+        <v>0.62</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>ANM2608CAROUEN000115</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>9648</v>
+      </c>
+      <c r="D85" t="b">
+        <v>1</v>
+      </c>
+      <c r="E85" t="n">
+        <v>9648.41</v>
+      </c>
+      <c r="F85" t="n">
+        <v>0</v>
+      </c>
+      <c r="G85" t="n">
+        <v>0</v>
+      </c>
+      <c r="H85" t="n">
+        <v>0</v>
+      </c>
+      <c r="I85" t="n">
+        <v>0</v>
+      </c>
+      <c r="J85" t="n">
+        <v>9648.41</v>
+      </c>
+      <c r="K85" t="n">
+        <v>0.41</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>ANM2608SGCASEN000239</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>1647.83</v>
+      </c>
+      <c r="D86" t="b">
+        <v>1</v>
+      </c>
+      <c r="E86" t="n">
+        <v>1648.17</v>
+      </c>
+      <c r="F86" t="n">
+        <v>0</v>
+      </c>
+      <c r="G86" t="n">
+        <v>0</v>
+      </c>
+      <c r="H86" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" t="n">
+        <v>0</v>
+      </c>
+      <c r="J86" t="n">
+        <v>1648.17</v>
+      </c>
+      <c r="K86" t="n">
+        <v>0.34</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>ANM2608SGMKCEN000016</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>75635.78</v>
+      </c>
+      <c r="D87" t="b">
+        <v>1</v>
+      </c>
+      <c r="E87" t="n">
+        <v>77106.7</v>
+      </c>
+      <c r="F87" t="n">
+        <v>0</v>
+      </c>
+      <c r="G87" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" t="n">
+        <v>0</v>
+      </c>
+      <c r="I87" t="n">
+        <v>1470.59</v>
+      </c>
+      <c r="J87" t="n">
+        <v>75636.11</v>
+      </c>
+      <c r="K87" t="n">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>ANM2608SGRBYEN000020</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>7219.61</v>
+      </c>
+      <c r="D88" t="b">
+        <v>1</v>
+      </c>
+      <c r="E88" t="n">
+        <v>7311.61</v>
+      </c>
+      <c r="F88" t="n">
+        <v>0</v>
+      </c>
+      <c r="G88" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" t="n">
+        <v>0</v>
+      </c>
+      <c r="I88" t="n">
+        <v>91.7</v>
+      </c>
+      <c r="J88" t="n">
+        <v>7219.91</v>
+      </c>
+      <c r="K88" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>ANM2608SGOUJEN000033</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>973994.78</v>
+      </c>
+      <c r="D89" t="b">
+        <v>1</v>
+      </c>
+      <c r="E89" t="n">
+        <v>973994.98</v>
+      </c>
+      <c r="F89" t="n">
+        <v>0</v>
+      </c>
+      <c r="G89" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" t="n">
+        <v>0</v>
+      </c>
+      <c r="I89" t="n">
+        <v>0</v>
+      </c>
+      <c r="J89" t="n">
+        <v>973994.98</v>
+      </c>
+      <c r="K89" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>ANM2608CARTGEN000068</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>8613</v>
+      </c>
+      <c r="D90" t="b">
+        <v>1</v>
+      </c>
+      <c r="E90" t="n">
+        <v>8613.15</v>
+      </c>
+      <c r="F90" t="n">
+        <v>0</v>
+      </c>
+      <c r="G90" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" t="n">
+        <v>0</v>
+      </c>
+      <c r="I90" t="n">
+        <v>0</v>
+      </c>
+      <c r="J90" t="n">
+        <v>8613.15</v>
+      </c>
+      <c r="K90" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>ANM2608AWCASEN000096</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>623516</v>
+      </c>
+      <c r="D91" t="b">
+        <v>1</v>
+      </c>
+      <c r="E91" t="n">
+        <v>623516.1</v>
+      </c>
+      <c r="F91" t="n">
+        <v>0</v>
+      </c>
+      <c r="G91" t="n">
+        <v>0</v>
+      </c>
+      <c r="H91" t="n">
+        <v>0</v>
+      </c>
+      <c r="I91" t="n">
+        <v>0</v>
+      </c>
+      <c r="J91" t="n">
+        <v>623516.1</v>
+      </c>
+      <c r="K91" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>ANM2608CARR2EN000114</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>404.21</v>
+      </c>
+      <c r="D92" t="b">
+        <v>1</v>
+      </c>
+      <c r="E92" t="n">
+        <v>404.28</v>
+      </c>
+      <c r="F92" t="n">
+        <v>0</v>
+      </c>
+      <c r="G92" t="n">
+        <v>0</v>
+      </c>
+      <c r="H92" t="n">
+        <v>0</v>
+      </c>
+      <c r="I92" t="n">
+        <v>0</v>
+      </c>
+      <c r="J92" t="n">
+        <v>404.28</v>
+      </c>
+      <c r="K92" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>ANM2608SGBVEN000039</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>19350.79</v>
+      </c>
+      <c r="D93" t="b">
+        <v>1</v>
+      </c>
+      <c r="E93" t="n">
+        <v>19596.57</v>
+      </c>
+      <c r="F93" t="n">
+        <v>0</v>
+      </c>
+      <c r="G93" t="n">
+        <v>0</v>
+      </c>
+      <c r="H93" t="n">
+        <v>0</v>
+      </c>
+      <c r="I93" t="n">
+        <v>245.74</v>
+      </c>
+      <c r="J93" t="n">
+        <v>19350.83</v>
+      </c>
+      <c r="K93" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
           <t>ANM2608SGRABEN000048</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>ENCAI</t>
-        </is>
-      </c>
-      <c r="C71" t="n">
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>ENCAI</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
         <v>42348.21</v>
       </c>
-      <c r="D71" t="b">
-        <v>1</v>
-      </c>
-      <c r="E71" t="n">
+      <c r="D94" t="b">
+        <v>1</v>
+      </c>
+      <c r="E94" t="n">
         <v>43168.04</v>
       </c>
-      <c r="F71" t="n">
-        <v>0</v>
-      </c>
-      <c r="G71" t="n">
-        <v>0</v>
-      </c>
-      <c r="H71" t="n">
-        <v>0</v>
-      </c>
-      <c r="I71" t="n">
+      <c r="F94" t="n">
+        <v>0</v>
+      </c>
+      <c r="G94" t="n">
+        <v>0</v>
+      </c>
+      <c r="H94" t="n">
+        <v>0</v>
+      </c>
+      <c r="I94" t="n">
         <v>819.79</v>
       </c>
-      <c r="J71" t="n">
+      <c r="J94" t="n">
         <v>42348.25</v>
       </c>
-      <c r="K71" t="n">
+      <c r="K94" t="n">
         <v>0.04</v>
       </c>
     </row>
@@ -4550,7 +5447,7 @@
         <v>1016163.35</v>
       </c>
       <c r="K31" t="n">
-        <v>0</v>
+        <v>2032326.7</v>
       </c>
     </row>
     <row r="32">
@@ -4589,7 +5486,7 @@
         <v>10750731.61</v>
       </c>
       <c r="K32" t="n">
-        <v>0</v>
+        <v>21501463.22</v>
       </c>
     </row>
     <row r="33">
@@ -4628,7 +5525,7 @@
         <v>41001305.23</v>
       </c>
       <c r="K33" t="n">
-        <v>0</v>
+        <v>82002610.45999999</v>
       </c>
     </row>
     <row r="34">
@@ -4667,7 +5564,7 @@
         <v>420846.76</v>
       </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>841693.52</v>
       </c>
     </row>
     <row r="35">
@@ -8684,7 +9581,7 @@
         <v>635968.0600000001</v>
       </c>
       <c r="K137" t="n">
-        <v>-557.91</v>
+        <v>1272494.03</v>
       </c>
     </row>
     <row r="138">
@@ -8723,7 +9620,7 @@
         <v>2121334.19</v>
       </c>
       <c r="K138" t="n">
-        <v>0</v>
+        <v>4242668.38</v>
       </c>
     </row>
     <row r="139">
@@ -8762,7 +9659,7 @@
         <v>90572.74000000001</v>
       </c>
       <c r="K139" t="n">
-        <v>0</v>
+        <v>181145.48</v>
       </c>
     </row>
     <row r="140">
@@ -8801,7 +9698,7 @@
         <v>318600.03</v>
       </c>
       <c r="K140" t="n">
-        <v>0</v>
+        <v>637200.0600000001</v>
       </c>
     </row>
     <row r="141">
@@ -8840,7 +9737,7 @@
         <v>12723617.12</v>
       </c>
       <c r="K141" t="n">
-        <v>0</v>
+        <v>25447234.24</v>
       </c>
     </row>
     <row r="142">
@@ -8879,7 +9776,7 @@
         <v>76566.37</v>
       </c>
       <c r="K142" t="n">
-        <v>-364.19</v>
+        <v>153496.93</v>
       </c>
     </row>
     <row r="143">
@@ -8918,7 +9815,7 @@
         <v>159876</v>
       </c>
       <c r="K143" t="n">
-        <v>-1404</v>
+        <v>321156</v>
       </c>
     </row>
     <row r="144">
@@ -8957,7 +9854,7 @@
         <v>6553.3</v>
       </c>
       <c r="K144" t="n">
-        <v>-26.92</v>
+        <v>13133.52</v>
       </c>
     </row>
     <row r="145">
@@ -8996,7 +9893,7 @@
         <v>12042309.91</v>
       </c>
       <c r="K145" t="n">
-        <v>0</v>
+        <v>24084619.82</v>
       </c>
     </row>
     <row r="146">
@@ -9035,7 +9932,7 @@
         <v>7491.29</v>
       </c>
       <c r="K146" t="n">
-        <v>0</v>
+        <v>14982.58</v>
       </c>
     </row>
     <row r="147">
@@ -9074,7 +9971,7 @@
         <v>8605.780000000001</v>
       </c>
       <c r="K147" t="n">
-        <v>0</v>
+        <v>17211.56</v>
       </c>
     </row>
     <row r="148">
@@ -9113,7 +10010,7 @@
         <v>48074.26</v>
       </c>
       <c r="K148" t="n">
-        <v>-381.81</v>
+        <v>96530.33</v>
       </c>
     </row>
     <row r="149">
@@ -9152,7 +10049,7 @@
         <v>13746148.84</v>
       </c>
       <c r="K149" t="n">
-        <v>0</v>
+        <v>27492297.68</v>
       </c>
     </row>
     <row r="150">
@@ -9191,7 +10088,7 @@
         <v>868428.23</v>
       </c>
       <c r="K150" t="n">
-        <v>0</v>
+        <v>1736856.46</v>
       </c>
     </row>
     <row r="151">
@@ -9230,7 +10127,7 @@
         <v>29165.74</v>
       </c>
       <c r="K151" t="n">
-        <v>-187.51</v>
+        <v>58518.99</v>
       </c>
     </row>
     <row r="152">
@@ -9269,7 +10166,7 @@
         <v>7096.65</v>
       </c>
       <c r="K152" t="n">
-        <v>-41.33</v>
+        <v>14234.63</v>
       </c>
     </row>
     <row r="153">
@@ -9308,7 +10205,7 @@
         <v>3217.98</v>
       </c>
       <c r="K153" t="n">
-        <v>-10.38</v>
+        <v>6446.34</v>
       </c>
     </row>
     <row r="154">
@@ -9347,7 +10244,7 @@
         <v>48473.94</v>
       </c>
       <c r="K154" t="n">
-        <v>0</v>
+        <v>96947.88</v>
       </c>
     </row>
     <row r="155">
@@ -9386,7 +10283,7 @@
         <v>251625.19</v>
       </c>
       <c r="K155" t="n">
-        <v>0</v>
+        <v>503250.38</v>
       </c>
     </row>
     <row r="156">
@@ -9425,7 +10322,7 @@
         <v>8706.559999999999</v>
       </c>
       <c r="K156" t="n">
-        <v>-105.22</v>
+        <v>17518.34</v>
       </c>
     </row>
     <row r="157">
@@ -9464,7 +10361,7 @@
         <v>47721.46</v>
       </c>
       <c r="K157" t="n">
-        <v>0</v>
+        <v>95442.92</v>
       </c>
     </row>
     <row r="158">
@@ -9503,7 +10400,7 @@
         <v>485172</v>
       </c>
       <c r="K158" t="n">
-        <v>0</v>
+        <v>970344</v>
       </c>
     </row>
     <row r="159">
@@ -9542,7 +10439,7 @@
         <v>60800.62</v>
       </c>
       <c r="K159" t="n">
-        <v>-115.74</v>
+        <v>121716.98</v>
       </c>
     </row>
     <row r="160">
@@ -9581,7 +10478,7 @@
         <v>112869.39</v>
       </c>
       <c r="K160" t="n">
-        <v>0</v>
+        <v>225738.78</v>
       </c>
     </row>
     <row r="161">
@@ -9620,7 +10517,7 @@
         <v>3370243.69</v>
       </c>
       <c r="K161" t="n">
-        <v>0</v>
+        <v>6740487.38</v>
       </c>
     </row>
     <row r="162">
@@ -9659,7 +10556,7 @@
         <v>177993.86</v>
       </c>
       <c r="K162" t="n">
-        <v>-1273.2</v>
+        <v>357260.92</v>
       </c>
     </row>
     <row r="163">
@@ -9698,7 +10595,7 @@
         <v>65245870.54</v>
       </c>
       <c r="K163" t="n">
-        <v>0</v>
+        <v>130491741.08</v>
       </c>
     </row>
     <row r="164">
@@ -83954,7 +84851,7 @@
         <v>20000</v>
       </c>
       <c r="K2067" t="n">
-        <v>0</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="2068">
@@ -90818,7 +91715,7 @@
         <v>5733574.23</v>
       </c>
       <c r="K2243" t="n">
-        <v>0</v>
+        <v>11467148.46</v>
       </c>
     </row>
     <row r="2244">
@@ -90857,7 +91754,7 @@
         <v>5448382.99</v>
       </c>
       <c r="K2244" t="n">
-        <v>-1293746.47</v>
+        <v>12190512.45</v>
       </c>
     </row>
     <row r="2245">
@@ -90896,7 +91793,7 @@
         <v>344512.34</v>
       </c>
       <c r="K2245" t="n">
-        <v>-1948.67</v>
+        <v>690973.35</v>
       </c>
     </row>
     <row r="2246">
@@ -91013,7 +91910,7 @@
         <v>7456</v>
       </c>
       <c r="K2248" t="n">
-        <v>0</v>
+        <v>14912</v>
       </c>
     </row>
     <row r="2249">
@@ -91325,7 +92222,7 @@
         <v>172341.31</v>
       </c>
       <c r="K2256" t="n">
-        <v>-1292.81</v>
+        <v>345975.43</v>
       </c>
     </row>
     <row r="2257">

</xml_diff>